<commit_message>
Fix practice exam PDF compilation
</commit_message>
<xml_diff>
--- a/banks/life-health/Module 1/Test Bank Reading - Org Forms.xlsx
+++ b/banks/life-health/Module 1/Test Bank Reading - Org Forms.xlsx
@@ -474,17 +474,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Specialization benefits &amp; agency conflicts to be managed</t>
+          <t>Specialization benefits \&amp; agency conflicts to be managed</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Guaranteed lower premiums &amp; zero insolvency risk</t>
+          <t>Guaranteed lower premiums \&amp; zero insolvency risk</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Perfectly aligned incentives &amp; faster claim payments</t>
+          <t>Perfectly aligned incentives \&amp; faster claim payments</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">

</xml_diff>